<commit_message>
Actualiza BD_Motos y regenera data.js
- Nueva version de BD_Motos (1344 modelos) -> mejor asignacion de marca
- Volumen reciente sin marca queda en 0.6%

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fuentes/BD_Motos.xlsx
+++ b/Fuentes/BD_Motos.xlsx
@@ -6,7 +6,7 @@
     <sheet state="visible" name="Consulta" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Consulta!$A$1:$C$1331</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Consulta!$A$1:$C$1370</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3961" uniqueCount="1438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4031" uniqueCount="1480">
   <si>
     <t>Marca</t>
   </si>
@@ -4332,6 +4332,132 @@
   </si>
   <si>
     <t>R1200 GS</t>
+  </si>
+  <si>
+    <t>Kymco</t>
+  </si>
+  <si>
+    <t>SKYTOWN 150</t>
+  </si>
+  <si>
+    <t>Kove</t>
+  </si>
+  <si>
+    <t>800X GT</t>
+  </si>
+  <si>
+    <t>Gilera</t>
+  </si>
+  <si>
+    <t>GC200 QUEEN</t>
+  </si>
+  <si>
+    <t>Keller</t>
+  </si>
+  <si>
+    <t>MX450 R</t>
+  </si>
+  <si>
+    <t>Honda / Genérico</t>
+  </si>
+  <si>
+    <t>CG 125</t>
+  </si>
+  <si>
+    <t>Mondial / Motomel</t>
+  </si>
+  <si>
+    <t>SL 125</t>
+  </si>
+  <si>
+    <t>KR260 A</t>
+  </si>
+  <si>
+    <t>Can-Am</t>
+  </si>
+  <si>
+    <t>RENEGADE 800 R</t>
+  </si>
+  <si>
+    <t>Benelli</t>
+  </si>
+  <si>
+    <t>STX150</t>
+  </si>
+  <si>
+    <t>TNT135</t>
+  </si>
+  <si>
+    <t>Yamaha</t>
+  </si>
+  <si>
+    <t>YFZ50</t>
+  </si>
+  <si>
+    <t>Kawasaki</t>
+  </si>
+  <si>
+    <t>NINJA H2</t>
+  </si>
+  <si>
+    <t>Nuuv</t>
+  </si>
+  <si>
+    <t>U PRO</t>
+  </si>
+  <si>
+    <t>RS300R</t>
+  </si>
+  <si>
+    <t>Beta</t>
+  </si>
+  <si>
+    <t>RR 125 2T</t>
+  </si>
+  <si>
+    <t>250 EXC-F SIX DAYS</t>
+  </si>
+  <si>
+    <t>Sunra</t>
+  </si>
+  <si>
+    <t>GRACE NXT 1</t>
+  </si>
+  <si>
+    <t>Ariic</t>
+  </si>
+  <si>
+    <t>ARIIC 318</t>
+  </si>
+  <si>
+    <t>Harley-Davidson</t>
+  </si>
+  <si>
+    <t>FLTRXSE CVO ROAD GLIDE</t>
+  </si>
+  <si>
+    <t>Husqvarna</t>
+  </si>
+  <si>
+    <t>TC 65</t>
+  </si>
+  <si>
+    <t>KLX450R</t>
+  </si>
+  <si>
+    <t>Corven</t>
+  </si>
+  <si>
+    <t>GRINDER</t>
+  </si>
+  <si>
+    <t>Voge</t>
+  </si>
+  <si>
+    <t>SR2 ADV</t>
+  </si>
+  <si>
+    <t>VOGE XWOLF 550L</t>
   </si>
 </sst>
 </file>
@@ -4366,9 +4492,9 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -4419,7 +4545,9 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -24429,105 +24557,302 @@
       <c r="G1321" s="5"/>
     </row>
     <row r="1322" ht="15.75" customHeight="1">
+      <c r="A1322" s="9" t="s">
+        <v>1438</v>
+      </c>
+      <c r="B1322" s="9" t="s">
+        <v>1439</v>
+      </c>
+      <c r="C1322" s="4" t="s">
+        <v>21</v>
+      </c>
       <c r="E1322" s="3"/>
       <c r="F1322" s="5"/>
       <c r="G1322" s="5"/>
     </row>
     <row r="1323" ht="15.75" customHeight="1">
-      <c r="A1323" s="9"/>
-      <c r="B1323" s="9"/>
-      <c r="C1323" s="9"/>
+      <c r="A1323" s="7" t="s">
+        <v>1440</v>
+      </c>
+      <c r="B1323" s="7" t="s">
+        <v>1441</v>
+      </c>
+      <c r="C1323" s="4" t="s">
+        <v>107</v>
+      </c>
       <c r="D1323" s="3"/>
       <c r="E1323" s="3"/>
       <c r="F1323" s="5"/>
       <c r="G1323" s="5"/>
     </row>
     <row r="1324" ht="15.75" customHeight="1">
-      <c r="A1324" s="9"/>
-      <c r="B1324" s="9"/>
-      <c r="C1324" s="9"/>
+      <c r="A1324" s="7" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B1324" s="7" t="s">
+        <v>1443</v>
+      </c>
+      <c r="C1324" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="D1324" s="3"/>
       <c r="E1324" s="3"/>
       <c r="F1324" s="5"/>
       <c r="G1324" s="5"/>
     </row>
     <row r="1325" ht="15.75" customHeight="1">
-      <c r="A1325" s="9"/>
-      <c r="B1325" s="9"/>
-      <c r="C1325" s="9"/>
+      <c r="A1325" s="7" t="s">
+        <v>1444</v>
+      </c>
+      <c r="B1325" s="9" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1325" s="4" t="s">
+        <v>107</v>
+      </c>
       <c r="D1325" s="3"/>
       <c r="E1325" s="3"/>
       <c r="F1325" s="5"/>
       <c r="G1325" s="5"/>
     </row>
     <row r="1326" ht="15.75" customHeight="1">
-      <c r="A1326" s="9"/>
-      <c r="B1326" s="9"/>
-      <c r="C1326" s="9"/>
+      <c r="A1326" s="7" t="s">
+        <v>1446</v>
+      </c>
+      <c r="B1326" s="9" t="s">
+        <v>1447</v>
+      </c>
+      <c r="C1326" s="4" t="s">
+        <v>21</v>
+      </c>
       <c r="D1326" s="3"/>
       <c r="E1326" s="3"/>
       <c r="F1326" s="5"/>
       <c r="G1326" s="5"/>
     </row>
     <row r="1327" ht="15.75" customHeight="1">
-      <c r="A1327" s="9"/>
-      <c r="B1327" s="9"/>
-      <c r="C1327" s="9"/>
+      <c r="A1327" s="7" t="s">
+        <v>1448</v>
+      </c>
+      <c r="B1327" s="9" t="s">
+        <v>1449</v>
+      </c>
+      <c r="C1327" s="4" t="s">
+        <v>21</v>
+      </c>
       <c r="D1327" s="3"/>
       <c r="E1327" s="3"/>
       <c r="F1327" s="5"/>
       <c r="G1327" s="5"/>
     </row>
     <row r="1328" ht="15.75" customHeight="1">
-      <c r="A1328" s="9"/>
-      <c r="B1328" s="9"/>
-      <c r="C1328" s="9"/>
+      <c r="A1328" s="7" t="s">
+        <v>1444</v>
+      </c>
+      <c r="B1328" s="9" t="s">
+        <v>1450</v>
+      </c>
+      <c r="C1328" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="D1328" s="3"/>
       <c r="E1328" s="3"/>
       <c r="F1328" s="5"/>
       <c r="G1328" s="5"/>
     </row>
     <row r="1329" ht="15.75" customHeight="1">
-      <c r="A1329" s="9"/>
-      <c r="B1329" s="9"/>
-      <c r="C1329" s="9"/>
+      <c r="A1329" s="7" t="s">
+        <v>1451</v>
+      </c>
+      <c r="B1329" s="9" t="s">
+        <v>1452</v>
+      </c>
+      <c r="C1329" s="4" t="s">
+        <v>107</v>
+      </c>
       <c r="D1329" s="3"/>
       <c r="E1329" s="3"/>
       <c r="F1329" s="5"/>
       <c r="G1329" s="5"/>
     </row>
     <row r="1330" ht="15.75" customHeight="1">
-      <c r="A1330" s="9"/>
-      <c r="B1330" s="9"/>
-      <c r="C1330" s="9"/>
+      <c r="A1330" s="7" t="s">
+        <v>1453</v>
+      </c>
+      <c r="B1330" s="9" t="s">
+        <v>1454</v>
+      </c>
+      <c r="C1330" s="4" t="s">
+        <v>21</v>
+      </c>
       <c r="D1330" s="3"/>
       <c r="E1330" s="3"/>
       <c r="F1330" s="5"/>
       <c r="G1330" s="5"/>
     </row>
     <row r="1331" ht="15.75" customHeight="1">
-      <c r="A1331" s="9"/>
-      <c r="B1331" s="9"/>
-      <c r="C1331" s="9"/>
+      <c r="A1331" s="9" t="s">
+        <v>1453</v>
+      </c>
+      <c r="B1331" s="9" t="s">
+        <v>1455</v>
+      </c>
+      <c r="C1331" s="4" t="s">
+        <v>21</v>
+      </c>
       <c r="D1331" s="3"/>
       <c r="E1331" s="3"/>
       <c r="F1331" s="5"/>
       <c r="G1331" s="5"/>
     </row>
-    <row r="1332" ht="15.75" customHeight="1"/>
-    <row r="1333" ht="15.75" customHeight="1"/>
-    <row r="1334" ht="15.75" customHeight="1"/>
-    <row r="1335" ht="15.75" customHeight="1"/>
-    <row r="1336" ht="15.75" customHeight="1"/>
-    <row r="1337" ht="15.75" customHeight="1"/>
-    <row r="1338" ht="15.75" customHeight="1"/>
-    <row r="1339" ht="15.75" customHeight="1"/>
-    <row r="1340" ht="15.75" customHeight="1"/>
-    <row r="1341" ht="15.75" customHeight="1"/>
-    <row r="1342" ht="15.75" customHeight="1"/>
-    <row r="1343" ht="15.75" customHeight="1"/>
-    <row r="1344" ht="15.75" customHeight="1"/>
-    <row r="1345" ht="15.75" customHeight="1"/>
+    <row r="1332" ht="15.75" customHeight="1">
+      <c r="A1332" s="9" t="s">
+        <v>1456</v>
+      </c>
+      <c r="B1332" s="9" t="s">
+        <v>1457</v>
+      </c>
+      <c r="C1332" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1333" ht="15.75" customHeight="1">
+      <c r="A1333" s="9" t="s">
+        <v>1458</v>
+      </c>
+      <c r="B1333" s="9" t="s">
+        <v>1459</v>
+      </c>
+      <c r="C1333" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="1334" ht="15.75" customHeight="1">
+      <c r="A1334" s="9" t="s">
+        <v>1460</v>
+      </c>
+      <c r="B1334" s="9" t="s">
+        <v>1461</v>
+      </c>
+    </row>
+    <row r="1335" ht="15.75" customHeight="1">
+      <c r="A1335" s="9" t="s">
+        <v>1389</v>
+      </c>
+      <c r="B1335" s="9" t="s">
+        <v>1462</v>
+      </c>
+      <c r="C1335" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1336" ht="15.75" customHeight="1">
+      <c r="A1336" s="9" t="s">
+        <v>1463</v>
+      </c>
+      <c r="B1336" s="9" t="s">
+        <v>1464</v>
+      </c>
+      <c r="C1336" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1337" ht="15.75" customHeight="1">
+      <c r="A1337" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1337" s="9" t="s">
+        <v>1465</v>
+      </c>
+      <c r="C1337" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1338" ht="15.75" customHeight="1">
+      <c r="A1338" s="9" t="s">
+        <v>1466</v>
+      </c>
+      <c r="B1338" s="9" t="s">
+        <v>1467</v>
+      </c>
+    </row>
+    <row r="1339" ht="15.75" customHeight="1">
+      <c r="A1339" s="9" t="s">
+        <v>1468</v>
+      </c>
+      <c r="B1339" s="9" t="s">
+        <v>1469</v>
+      </c>
+      <c r="C1339" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1340" ht="15.75" customHeight="1">
+      <c r="A1340" s="9" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B1340" s="9" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C1340" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="1341" ht="15.75" customHeight="1">
+      <c r="A1341" s="9" t="s">
+        <v>1472</v>
+      </c>
+      <c r="B1341" s="9" t="s">
+        <v>1473</v>
+      </c>
+      <c r="C1341" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1342" ht="15.75" customHeight="1">
+      <c r="A1342" s="9" t="s">
+        <v>1458</v>
+      </c>
+      <c r="B1342" s="9" t="s">
+        <v>1474</v>
+      </c>
+      <c r="C1342" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1343" ht="15.75" customHeight="1">
+      <c r="A1343" s="9" t="s">
+        <v>1475</v>
+      </c>
+      <c r="B1343" s="9" t="s">
+        <v>1476</v>
+      </c>
+      <c r="C1343" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1344" ht="15.75" customHeight="1">
+      <c r="A1344" s="9" t="s">
+        <v>1477</v>
+      </c>
+      <c r="B1344" s="9" t="s">
+        <v>1478</v>
+      </c>
+      <c r="C1344" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1345" ht="15.75" customHeight="1">
+      <c r="A1345" s="9" t="s">
+        <v>1477</v>
+      </c>
+      <c r="B1345" s="9" t="s">
+        <v>1479</v>
+      </c>
+      <c r="C1345" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
     <row r="1346" ht="15.75" customHeight="1"/>
     <row r="1347" ht="15.75" customHeight="1"/>
     <row r="1348" ht="15.75" customHeight="1"/>
@@ -31378,7 +31703,7 @@
     <row r="8193" ht="15.75" customHeight="1"/>
     <row r="8194" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$1:$C$1331"/>
+  <autoFilter ref="$A$1:$C$1370"/>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>